<commit_message>
[ADD] Forward search plots
</commit_message>
<xml_diff>
--- a/results/greedy_params_choice_splashing_300iters.xlsx
+++ b/results/greedy_params_choice_splashing_300iters.xlsx
@@ -699,7 +699,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'K', 'inclination', 'volume_fraction', 'wettability')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'K', 'sedimentation_Stk', 'wettability', 'inclination')</t>
         </is>
       </c>
       <c r="I2" t="n">
@@ -881,7 +881,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'K', 'inclination', 'volume_fraction', 'wettability')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'K', 'sedimentation_Stk', 'wettability', 'inclination')</t>
         </is>
       </c>
       <c r="I3" t="n">
@@ -1063,7 +1063,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'relative_roughness', 'particle_droplet_diameter_ratio', 'K', 'inclination', 'volume_fraction', 'wettability')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'K', 'wettability', 'inclination', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I4" t="n">
@@ -1245,7 +1245,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'relative_roughness', 'particle_droplet_diameter_ratio', 'K', 'inclination', 'volume_fraction', 'wettability')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'K', 'wettability', 'inclination', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'relative_roughness', 'sedimentation_Stk', 'K', 'inclination', 'volume_fraction', 'wettability')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'K', 'sedimentation_Stk', 'wettability', 'inclination', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -1609,7 +1609,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'relative_roughness', 'sedimentation_Stk', 'K', 'inclination', 'volume_fraction', 'wettability')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'K', 'sedimentation_Stk', 'wettability', 'inclination', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -1791,7 +1791,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'relative_roughness', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'K', 'volume_fraction', 'wettability')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'K', 'sedimentation_Stk', 'wettability', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -1973,7 +1973,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'relative_roughness', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'K', 'volume_fraction', 'wettability')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'K', 'sedimentation_Stk', 'wettability', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -2155,7 +2155,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'relative_roughness', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'K', 'inclination', 'wettability')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'K', 'sedimentation_Stk', 'wettability', 'inclination', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -2337,7 +2337,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'relative_roughness', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'K', 'inclination', 'wettability')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'K', 'sedimentation_Stk', 'wettability', 'inclination', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -2519,7 +2519,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'relative_roughness', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'K', 'inclination', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'K', 'sedimentation_Stk', 'inclination', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -2699,7 +2699,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'relative_roughness', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'K', 'inclination', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'K', 'sedimentation_Stk', 'inclination', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -2881,7 +2881,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'relative_roughness', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'inclination', 'volume_fraction', 'wettability')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'wettability', 'inclination', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -3063,7 +3063,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'relative_roughness', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'inclination', 'volume_fraction', 'wettability')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'wettability', 'inclination', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -3245,7 +3245,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'K', 'inclination', 'volume_fraction', 'wettability')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'K', 'wettability', 'inclination')</t>
         </is>
       </c>
       <c r="I16" t="n">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'K', 'inclination', 'volume_fraction', 'wettability')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'K', 'wettability', 'inclination')</t>
         </is>
       </c>
       <c r="I17" t="n">
@@ -3609,7 +3609,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'K', 'inclination', 'volume_fraction', 'wettability')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'K', 'sedimentation_Stk', 'wettability', 'inclination')</t>
         </is>
       </c>
       <c r="I18" t="n">
@@ -3791,7 +3791,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'K', 'inclination', 'volume_fraction', 'wettability')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'K', 'sedimentation_Stk', 'wettability', 'inclination')</t>
         </is>
       </c>
       <c r="I19" t="n">
@@ -3973,7 +3973,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'K', 'volume_fraction', 'wettability')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'K', 'sedimentation_Stk', 'wettability')</t>
         </is>
       </c>
       <c r="I20" t="n">
@@ -4155,7 +4155,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'K', 'volume_fraction', 'wettability')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'K', 'sedimentation_Stk', 'wettability')</t>
         </is>
       </c>
       <c r="I21" t="n">
@@ -4337,7 +4337,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'K', 'inclination', 'wettability')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'K', 'sedimentation_Stk', 'wettability', 'inclination')</t>
         </is>
       </c>
       <c r="I22" t="n">
@@ -4519,7 +4519,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'K', 'inclination', 'wettability')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'K', 'sedimentation_Stk', 'wettability', 'inclination')</t>
         </is>
       </c>
       <c r="I23" t="n">
@@ -4701,7 +4701,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'K', 'inclination', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'K', 'sedimentation_Stk', 'inclination')</t>
         </is>
       </c>
       <c r="I24" t="n">
@@ -4883,7 +4883,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'K', 'inclination', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'K', 'sedimentation_Stk', 'inclination')</t>
         </is>
       </c>
       <c r="I25" t="n">
@@ -5065,7 +5065,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'inclination', 'volume_fraction', 'wettability')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'wettability', 'inclination')</t>
         </is>
       </c>
       <c r="I26" t="n">
@@ -5247,7 +5247,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'inclination', 'volume_fraction', 'wettability')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'wettability', 'inclination')</t>
         </is>
       </c>
       <c r="I27" t="n">
@@ -5429,7 +5429,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'relative_roughness', 'K', 'inclination', 'volume_fraction', 'wettability')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'K', 'wettability', 'inclination', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I28" t="n">
@@ -5611,7 +5611,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'relative_roughness', 'K', 'inclination', 'volume_fraction', 'wettability')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'K', 'wettability', 'inclination', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I29" t="n">
@@ -5793,7 +5793,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'relative_roughness', 'particle_droplet_diameter_ratio', 'K', 'volume_fraction', 'wettability')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'K', 'wettability', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I30" t="n">
@@ -5975,7 +5975,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'relative_roughness', 'particle_droplet_diameter_ratio', 'K', 'volume_fraction', 'wettability')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'K', 'wettability', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I31" t="n">
@@ -6157,7 +6157,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'relative_roughness', 'particle_droplet_diameter_ratio', 'K', 'inclination', 'wettability')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'K', 'wettability', 'inclination', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I32" t="n">
@@ -6339,7 +6339,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'relative_roughness', 'particle_droplet_diameter_ratio', 'K', 'inclination', 'wettability')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'K', 'wettability', 'inclination', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I33" t="n">
@@ -6521,7 +6521,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'relative_roughness', 'particle_droplet_diameter_ratio', 'K', 'inclination', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'K', 'inclination', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I34" t="n">
@@ -6703,7 +6703,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'relative_roughness', 'particle_droplet_diameter_ratio', 'K', 'inclination', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'K', 'inclination', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I35" t="n">
@@ -6885,7 +6885,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'relative_roughness', 'particle_droplet_diameter_ratio', 'inclination', 'volume_fraction', 'wettability')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'wettability', 'inclination', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I36" t="n">
@@ -7067,7 +7067,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'relative_roughness', 'particle_droplet_diameter_ratio', 'inclination', 'volume_fraction', 'wettability')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'wettability', 'inclination', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I37" t="n">
@@ -7249,7 +7249,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'relative_roughness', 'sedimentation_Stk', 'K', 'volume_fraction', 'wettability')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'K', 'sedimentation_Stk', 'wettability', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I38" t="n">
@@ -7431,7 +7431,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'relative_roughness', 'sedimentation_Stk', 'K', 'volume_fraction', 'wettability')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'K', 'sedimentation_Stk', 'wettability', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I39" t="n">
@@ -7613,7 +7613,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'relative_roughness', 'sedimentation_Stk', 'K', 'inclination', 'wettability')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'K', 'sedimentation_Stk', 'wettability', 'inclination', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I40" t="n">
@@ -7795,7 +7795,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'relative_roughness', 'sedimentation_Stk', 'K', 'inclination', 'wettability')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'K', 'sedimentation_Stk', 'wettability', 'inclination', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I41" t="n">
@@ -7977,7 +7977,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'relative_roughness', 'sedimentation_Stk', 'K', 'inclination', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'K', 'sedimentation_Stk', 'inclination', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I42" t="n">
@@ -8159,7 +8159,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'relative_roughness', 'sedimentation_Stk', 'K', 'inclination', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'K', 'sedimentation_Stk', 'inclination', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I43" t="n">
@@ -8341,7 +8341,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'relative_roughness', 'sedimentation_Stk', 'inclination', 'volume_fraction', 'wettability')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'sedimentation_Stk', 'wettability', 'inclination', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I44" t="n">
@@ -8523,7 +8523,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'relative_roughness', 'sedimentation_Stk', 'inclination', 'volume_fraction', 'wettability')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'sedimentation_Stk', 'wettability', 'inclination', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I45" t="n">
@@ -8705,7 +8705,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'relative_roughness', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'K', 'wettability')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'K', 'sedimentation_Stk', 'wettability', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I46" t="n">
@@ -8887,7 +8887,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'relative_roughness', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'K', 'wettability')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'K', 'sedimentation_Stk', 'wettability', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I47" t="n">
@@ -9069,7 +9069,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'relative_roughness', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'K', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'K', 'sedimentation_Stk', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I48" t="n">
@@ -9251,7 +9251,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'relative_roughness', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'K', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'K', 'sedimentation_Stk', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I49" t="n">
@@ -9433,7 +9433,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'relative_roughness', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'volume_fraction', 'wettability')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'wettability', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I50" t="n">
@@ -9615,7 +9615,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'relative_roughness', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'volume_fraction', 'wettability')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'wettability', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I51" t="n">
@@ -9797,7 +9797,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'relative_roughness', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'K', 'inclination')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'K', 'sedimentation_Stk', 'inclination', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I52" t="n">
@@ -9979,7 +9979,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'relative_roughness', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'K', 'inclination')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'K', 'sedimentation_Stk', 'inclination', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I53" t="n">
@@ -10161,7 +10161,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'relative_roughness', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'inclination', 'wettability')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'wettability', 'inclination', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I54" t="n">
@@ -10343,7 +10343,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'relative_roughness', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'inclination', 'wettability')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'wettability', 'inclination', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I55" t="n">
@@ -10525,7 +10525,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'relative_roughness', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'inclination', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'inclination', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I56" t="n">
@@ -10707,7 +10707,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'relative_roughness', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'inclination', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'inclination', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I57" t="n">
@@ -10889,7 +10889,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'K', 'inclination', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'volume_fraction', 'inclination', 'K')</t>
         </is>
       </c>
       <c r="I58" t="n">
@@ -11071,7 +11071,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'K', 'inclination', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'volume_fraction', 'inclination', 'K')</t>
         </is>
       </c>
       <c r="I59" t="n">
@@ -11253,7 +11253,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'particle_droplet_diameter_ratio', 'K', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'wettability', 'particle_droplet_diameter_ratio', 'K')</t>
         </is>
       </c>
       <c r="I60" t="n">
@@ -11435,7 +11435,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'particle_droplet_diameter_ratio', 'K', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'wettability', 'particle_droplet_diameter_ratio', 'K')</t>
         </is>
       </c>
       <c r="I61" t="n">
@@ -11617,7 +11617,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'particle_droplet_diameter_ratio', 'K', 'inclination')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'particle_droplet_diameter_ratio', 'inclination', 'K')</t>
         </is>
       </c>
       <c r="I62" t="n">
@@ -11799,7 +11799,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'particle_droplet_diameter_ratio', 'K', 'inclination')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'particle_droplet_diameter_ratio', 'inclination', 'K')</t>
         </is>
       </c>
       <c r="I63" t="n">
@@ -11981,7 +11981,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'K', 'inclination', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'inclination', 'K')</t>
         </is>
       </c>
       <c r="I64" t="n">
@@ -12163,7 +12163,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'K', 'inclination', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'inclination', 'K')</t>
         </is>
       </c>
       <c r="I65" t="n">
@@ -12345,7 +12345,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'particle_droplet_diameter_ratio', 'inclination', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'wettability', 'particle_droplet_diameter_ratio', 'inclination')</t>
         </is>
       </c>
       <c r="I66" t="n">
@@ -12527,7 +12527,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'particle_droplet_diameter_ratio', 'inclination', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'wettability', 'particle_droplet_diameter_ratio', 'inclination')</t>
         </is>
       </c>
       <c r="I67" t="n">
@@ -12709,7 +12709,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'sedimentation_Stk', 'K', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'wettability', 'volume_fraction', 'K')</t>
         </is>
       </c>
       <c r="I68" t="n">
@@ -12891,7 +12891,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'sedimentation_Stk', 'K', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'wettability', 'volume_fraction', 'K')</t>
         </is>
       </c>
       <c r="I69" t="n">
@@ -13073,7 +13073,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'sedimentation_Stk', 'K', 'inclination')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'wettability', 'K', 'inclination')</t>
         </is>
       </c>
       <c r="I70" t="n">
@@ -13255,7 +13255,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'sedimentation_Stk', 'K', 'inclination')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'wettability', 'K', 'inclination')</t>
         </is>
       </c>
       <c r="I71" t="n">
@@ -13437,7 +13437,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'inclination', 'sedimentation_Stk', 'K', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'volume_fraction', 'inclination', 'K')</t>
         </is>
       </c>
       <c r="I72" t="n">
@@ -13619,7 +13619,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'inclination', 'sedimentation_Stk', 'K', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'volume_fraction', 'inclination', 'K')</t>
         </is>
       </c>
       <c r="I73" t="n">
@@ -13801,7 +13801,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'sedimentation_Stk', 'inclination', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'wettability', 'volume_fraction', 'inclination')</t>
         </is>
       </c>
       <c r="I74" t="n">
@@ -13983,7 +13983,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'sedimentation_Stk', 'inclination', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'wettability', 'volume_fraction', 'inclination')</t>
         </is>
       </c>
       <c r="I75" t="n">
@@ -14165,7 +14165,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'sedimentation_Stk', 'particle_droplet_diameter_ratio', 'K')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'wettability', 'particle_droplet_diameter_ratio', 'K')</t>
         </is>
       </c>
       <c r="I76" t="n">
@@ -14347,7 +14347,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'sedimentation_Stk', 'particle_droplet_diameter_ratio', 'K')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'wettability', 'particle_droplet_diameter_ratio', 'K')</t>
         </is>
       </c>
       <c r="I77" t="n">
@@ -14529,7 +14529,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'K', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'K', 'sedimentation_Stk')</t>
         </is>
       </c>
       <c r="I78" t="n">
@@ -14711,7 +14711,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'K', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'K', 'sedimentation_Stk')</t>
         </is>
       </c>
       <c r="I79" t="n">
@@ -14893,7 +14893,7 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'sedimentation_Stk', 'particle_droplet_diameter_ratio', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'wettability', 'particle_droplet_diameter_ratio', 'sedimentation_Stk')</t>
         </is>
       </c>
       <c r="I80" t="n">
@@ -15075,7 +15075,7 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'sedimentation_Stk', 'particle_droplet_diameter_ratio', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'wettability', 'particle_droplet_diameter_ratio', 'sedimentation_Stk')</t>
         </is>
       </c>
       <c r="I81" t="n">
@@ -15257,7 +15257,7 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'K', 'inclination')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'particle_droplet_diameter_ratio', 'inclination', 'K')</t>
         </is>
       </c>
       <c r="I82" t="n">
@@ -15439,7 +15439,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'K', 'inclination')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'particle_droplet_diameter_ratio', 'inclination', 'K')</t>
         </is>
       </c>
       <c r="I83" t="n">
@@ -15621,7 +15621,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'sedimentation_Stk', 'particle_droplet_diameter_ratio', 'inclination')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'wettability', 'particle_droplet_diameter_ratio', 'inclination')</t>
         </is>
       </c>
       <c r="I84" t="n">
@@ -15803,7 +15803,7 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'sedimentation_Stk', 'particle_droplet_diameter_ratio', 'inclination')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'wettability', 'particle_droplet_diameter_ratio', 'inclination')</t>
         </is>
       </c>
       <c r="I85" t="n">
@@ -15985,7 +15985,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'inclination', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'inclination', 'sedimentation_Stk')</t>
         </is>
       </c>
       <c r="I86" t="n">
@@ -16167,7 +16167,7 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'inclination', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'inclination', 'sedimentation_Stk')</t>
         </is>
       </c>
       <c r="I87" t="n">
@@ -16349,7 +16349,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'K', 'volume_fraction', 'relative_roughness')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'volume_fraction', 'K', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I88" t="n">
@@ -16531,7 +16531,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'K', 'volume_fraction', 'relative_roughness')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'volume_fraction', 'K', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I89" t="n">
@@ -17077,7 +17077,7 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'inclination', 'K', 'volume_fraction', 'relative_roughness')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'inclination', 'K', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I92" t="n">
@@ -17259,7 +17259,7 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'inclination', 'K', 'volume_fraction', 'relative_roughness')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'inclination', 'K', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I93" t="n">
@@ -17441,7 +17441,7 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'inclination', 'volume_fraction', 'relative_roughness')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'volume_fraction', 'inclination', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I94" t="n">
@@ -17623,7 +17623,7 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'inclination', 'volume_fraction', 'relative_roughness')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'volume_fraction', 'inclination', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I95" t="n">
@@ -18169,7 +18169,7 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'K', 'volume_fraction', 'relative_roughness')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'K', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I98" t="n">
@@ -18351,7 +18351,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'K', 'volume_fraction', 'relative_roughness')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'K', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I99" t="n">
@@ -18533,7 +18533,7 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'particle_droplet_diameter_ratio', 'volume_fraction', 'relative_roughness')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'wettability', 'particle_droplet_diameter_ratio', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I100" t="n">
@@ -18715,7 +18715,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'particle_droplet_diameter_ratio', 'volume_fraction', 'relative_roughness')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'wettability', 'particle_droplet_diameter_ratio', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I101" t="n">
@@ -18897,7 +18897,7 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'K', 'inclination', 'relative_roughness')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'inclination', 'K', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I102" t="n">
@@ -19079,7 +19079,7 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'K', 'inclination', 'relative_roughness')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'inclination', 'K', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I103" t="n">
@@ -19625,7 +19625,7 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'inclination', 'volume_fraction', 'relative_roughness')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'inclination', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I106" t="n">
@@ -19807,7 +19807,7 @@
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'inclination', 'volume_fraction', 'relative_roughness')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'inclination', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I107" t="n">
@@ -19989,7 +19989,7 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'sedimentation_Stk', 'K', 'relative_roughness')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'wettability', 'K', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I108" t="n">
@@ -20171,7 +20171,7 @@
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'sedimentation_Stk', 'K', 'relative_roughness')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'wettability', 'K', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I109" t="n">
@@ -20353,7 +20353,7 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'sedimentation_Stk', 'K', 'relative_roughness')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'volume_fraction', 'K', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I110" t="n">
@@ -20535,7 +20535,7 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'sedimentation_Stk', 'K', 'relative_roughness')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'volume_fraction', 'K', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I111" t="n">
@@ -20717,7 +20717,7 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'sedimentation_Stk', 'volume_fraction', 'relative_roughness')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'wettability', 'volume_fraction', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I112" t="n">
@@ -20899,7 +20899,7 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'sedimentation_Stk', 'volume_fraction', 'relative_roughness')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'wettability', 'volume_fraction', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I113" t="n">
@@ -21081,7 +21081,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'inclination', 'sedimentation_Stk', 'K', 'relative_roughness')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'K', 'inclination', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I114" t="n">
@@ -21263,7 +21263,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'inclination', 'sedimentation_Stk', 'K', 'relative_roughness')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'K', 'inclination', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I115" t="n">
@@ -21445,7 +21445,7 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'sedimentation_Stk', 'inclination', 'relative_roughness')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'wettability', 'inclination', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I116" t="n">
@@ -21627,7 +21627,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'sedimentation_Stk', 'inclination', 'relative_roughness')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'wettability', 'inclination', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I117" t="n">
@@ -21809,7 +21809,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'sedimentation_Stk', 'inclination', 'relative_roughness')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'volume_fraction', 'inclination', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I118" t="n">
@@ -21991,7 +21991,7 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'sedimentation_Stk', 'inclination', 'relative_roughness')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'volume_fraction', 'inclination', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I119" t="n">
@@ -22173,7 +22173,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'K', 'relative_roughness')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'particle_droplet_diameter_ratio', 'K', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I120" t="n">
@@ -22355,7 +22355,7 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'K', 'relative_roughness')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'particle_droplet_diameter_ratio', 'K', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I121" t="n">
@@ -22537,7 +22537,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'wettability', 'particle_droplet_diameter_ratio', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I122" t="n">
@@ -22719,7 +22719,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'wettability', 'particle_droplet_diameter_ratio', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I123" t="n">
@@ -22901,7 +22901,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'volume_fraction', 'relative_roughness')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'relative_roughness', 'sedimentation_Stk')</t>
         </is>
       </c>
       <c r="I124" t="n">
@@ -23083,7 +23083,7 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'volume_fraction', 'relative_roughness')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'relative_roughness', 'sedimentation_Stk')</t>
         </is>
       </c>
       <c r="I125" t="n">
@@ -23265,7 +23265,7 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'inclination', 'relative_roughness')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'particle_droplet_diameter_ratio', 'inclination', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I126" t="n">
@@ -23447,7 +23447,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'inclination', 'relative_roughness')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'particle_droplet_diameter_ratio', 'inclination', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I127" t="n">
@@ -23629,7 +23629,7 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'K', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'volume_fraction', 'K')</t>
         </is>
       </c>
       <c r="I128" t="n">
@@ -23811,7 +23811,7 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'K', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'volume_fraction', 'K')</t>
         </is>
       </c>
       <c r="I129" t="n">
@@ -24357,7 +24357,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'inclination', 'K', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'inclination', 'K')</t>
         </is>
       </c>
       <c r="I132" t="n">
@@ -24539,7 +24539,7 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'inclination', 'K', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'inclination', 'K')</t>
         </is>
       </c>
       <c r="I133" t="n">
@@ -24721,7 +24721,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'inclination', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'volume_fraction', 'inclination')</t>
         </is>
       </c>
       <c r="I134" t="n">
@@ -24903,7 +24903,7 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'inclination', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'volume_fraction', 'inclination')</t>
         </is>
       </c>
       <c r="I135" t="n">
@@ -25449,7 +25449,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'K', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'K')</t>
         </is>
       </c>
       <c r="I138" t="n">
@@ -25631,7 +25631,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'K', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'K')</t>
         </is>
       </c>
       <c r="I139" t="n">
@@ -25813,7 +25813,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'particle_droplet_diameter_ratio', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'wettability', 'particle_droplet_diameter_ratio')</t>
         </is>
       </c>
       <c r="I140" t="n">
@@ -25995,7 +25995,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'particle_droplet_diameter_ratio', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'wettability', 'particle_droplet_diameter_ratio')</t>
         </is>
       </c>
       <c r="I141" t="n">
@@ -26177,7 +26177,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'K', 'inclination')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'inclination', 'K')</t>
         </is>
       </c>
       <c r="I142" t="n">
@@ -26359,7 +26359,7 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'K', 'inclination')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'inclination', 'K')</t>
         </is>
       </c>
       <c r="I143" t="n">
@@ -26905,7 +26905,7 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'inclination', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'inclination')</t>
         </is>
       </c>
       <c r="I146" t="n">
@@ -27087,7 +27087,7 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'inclination', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'inclination')</t>
         </is>
       </c>
       <c r="I147" t="n">
@@ -27269,7 +27269,7 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'sedimentation_Stk', 'K')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'wettability', 'K')</t>
         </is>
       </c>
       <c r="I148" t="n">
@@ -27451,7 +27451,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'sedimentation_Stk', 'K')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'wettability', 'K')</t>
         </is>
       </c>
       <c r="I149" t="n">
@@ -27633,7 +27633,7 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'sedimentation_Stk', 'K')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'volume_fraction', 'K')</t>
         </is>
       </c>
       <c r="I150" t="n">
@@ -27815,7 +27815,7 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'sedimentation_Stk', 'K')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'volume_fraction', 'K')</t>
         </is>
       </c>
       <c r="I151" t="n">
@@ -27997,7 +27997,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'sedimentation_Stk', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'wettability', 'volume_fraction')</t>
         </is>
       </c>
       <c r="I152" t="n">
@@ -28179,7 +28179,7 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'sedimentation_Stk', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'wettability', 'volume_fraction')</t>
         </is>
       </c>
       <c r="I153" t="n">
@@ -28361,7 +28361,7 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'inclination', 'sedimentation_Stk', 'K')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'K', 'inclination')</t>
         </is>
       </c>
       <c r="I154" t="n">
@@ -28543,7 +28543,7 @@
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'inclination', 'sedimentation_Stk', 'K')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'K', 'inclination')</t>
         </is>
       </c>
       <c r="I155" t="n">
@@ -28725,7 +28725,7 @@
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'sedimentation_Stk', 'inclination')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'wettability', 'inclination')</t>
         </is>
       </c>
       <c r="I156" t="n">
@@ -28907,7 +28907,7 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'sedimentation_Stk', 'inclination')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'wettability', 'inclination')</t>
         </is>
       </c>
       <c r="I157" t="n">
@@ -29089,7 +29089,7 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'sedimentation_Stk', 'inclination')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'volume_fraction', 'inclination')</t>
         </is>
       </c>
       <c r="I158" t="n">
@@ -29271,7 +29271,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'sedimentation_Stk', 'inclination')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'volume_fraction', 'inclination')</t>
         </is>
       </c>
       <c r="I159" t="n">
@@ -29453,7 +29453,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'K')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'particle_droplet_diameter_ratio', 'K')</t>
         </is>
       </c>
       <c r="I160" t="n">
@@ -29635,7 +29635,7 @@
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'K')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'particle_droplet_diameter_ratio', 'K')</t>
         </is>
       </c>
       <c r="I161" t="n">
@@ -29817,7 +29817,7 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'sedimentation_Stk', 'particle_droplet_diameter_ratio')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'wettability', 'particle_droplet_diameter_ratio')</t>
         </is>
       </c>
       <c r="I162" t="n">
@@ -29999,7 +29999,7 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'sedimentation_Stk', 'particle_droplet_diameter_ratio')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'wettability', 'particle_droplet_diameter_ratio')</t>
         </is>
       </c>
       <c r="I163" t="n">
@@ -30181,7 +30181,7 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'sedimentation_Stk')</t>
         </is>
       </c>
       <c r="I164" t="n">
@@ -30363,7 +30363,7 @@
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'sedimentation_Stk')</t>
         </is>
       </c>
       <c r="I165" t="n">
@@ -30545,7 +30545,7 @@
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'inclination')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'particle_droplet_diameter_ratio', 'inclination')</t>
         </is>
       </c>
       <c r="I166" t="n">
@@ -30727,7 +30727,7 @@
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'inclination')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'particle_droplet_diameter_ratio', 'inclination')</t>
         </is>
       </c>
       <c r="I167" t="n">
@@ -32001,7 +32001,7 @@
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'inclination', 'K', 'relative_roughness')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'K', 'inclination', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I174" t="n">
@@ -32183,7 +32183,7 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'inclination', 'K', 'relative_roughness')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'K', 'inclination', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I175" t="n">
@@ -33821,7 +33821,7 @@
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'volume_fraction', 'relative_roughness')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I184" t="n">
@@ -34003,7 +34003,7 @@
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'volume_fraction', 'relative_roughness')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I185" t="n">
@@ -34913,7 +34913,7 @@
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'sedimentation_Stk', 'relative_roughness')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'wettability', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I190" t="n">
@@ -35095,7 +35095,7 @@
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'sedimentation_Stk', 'relative_roughness')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'wettability', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I191" t="n">
@@ -35277,7 +35277,7 @@
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'sedimentation_Stk', 'relative_roughness')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'volume_fraction', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I192" t="n">
@@ -35459,7 +35459,7 @@
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'sedimentation_Stk', 'relative_roughness')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'volume_fraction', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I193" t="n">
@@ -36005,7 +36005,7 @@
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'relative_roughness')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I196" t="n">
@@ -36187,7 +36187,7 @@
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'sedimentation_Stk', 'relative_roughness')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness')</t>
         </is>
       </c>
       <c r="I197" t="n">
@@ -37461,7 +37461,7 @@
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'inclination', 'K')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'K', 'inclination')</t>
         </is>
       </c>
       <c r="I204" t="n">
@@ -37643,7 +37643,7 @@
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'inclination', 'K')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'K', 'inclination')</t>
         </is>
       </c>
       <c r="I205" t="n">
@@ -39281,7 +39281,7 @@
       </c>
       <c r="H214" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio')</t>
         </is>
       </c>
       <c r="I214" t="n">
@@ -39463,7 +39463,7 @@
       </c>
       <c r="H215" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'volume_fraction')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'particle_droplet_diameter_ratio')</t>
         </is>
       </c>
       <c r="I215" t="n">
@@ -40373,7 +40373,7 @@
       </c>
       <c r="H220" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'sedimentation_Stk')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'wettability')</t>
         </is>
       </c>
       <c r="I220" t="n">
@@ -40555,7 +40555,7 @@
       </c>
       <c r="H221" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'wettability', 'sedimentation_Stk')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'wettability')</t>
         </is>
       </c>
       <c r="I221" t="n">
@@ -40737,7 +40737,7 @@
       </c>
       <c r="H222" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'sedimentation_Stk')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'volume_fraction')</t>
         </is>
       </c>
       <c r="I222" t="n">
@@ -40919,7 +40919,7 @@
       </c>
       <c r="H223" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'volume_fraction', 'sedimentation_Stk')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'volume_fraction')</t>
         </is>
       </c>
       <c r="I223" t="n">
@@ -41465,7 +41465,7 @@
       </c>
       <c r="H226" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'sedimentation_Stk')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'particle_droplet_diameter_ratio')</t>
         </is>
       </c>
       <c r="I226" t="n">
@@ -41647,7 +41647,7 @@
       </c>
       <c r="H227" t="inlineStr">
         <is>
-          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'particle_droplet_diameter_ratio', 'sedimentation_Stk')</t>
+          <t>('sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Stk', 'Re', 'We', 'init_volume_fraction', 'sedimentation_Re', 'particle_liquid_density_ratio', 'sign_sedimentation_Re', 'sedimentation_Stk', 'particle_droplet_diameter_ratio')</t>
         </is>
       </c>
       <c r="I227" t="n">

</xml_diff>